<commit_message>
feat: update analysis data and add new draft sections file
Updated position bias summary CSV with corrected model scoring method labels, refreshed metrics and hybrid ablation Excel files with latest results, and added paper/draft_sections_new_analyses.tex to .gitignore.
</commit_message>
<xml_diff>
--- a/Analysis/MetricsSummary/metrics_summary_all_models.xlsx
+++ b/Analysis/MetricsSummary/metrics_summary_all_models.xlsx
@@ -560,7 +560,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.1656</v>
+        <v>0.1676</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -585,7 +585,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.2067</v>
+        <v>0.2084</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -660,7 +660,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.2076</v>
+        <v>0.2081</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.2714</v>
+        <v>0.2718</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>1.3073</v>
+        <v>1.3061</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -810,7 +810,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>1</v>
+        <v>0.7179</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -1210,7 +1210,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>1</v>
+        <v>0.6714</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1610,7 +1610,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>1</v>
+        <v>0.5538</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1760,7 +1760,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>0.1778</v>
+        <v>0.1843</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1785,7 +1785,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>0.2244</v>
+        <v>0.2294</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1860,7 +1860,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>0.1809</v>
+        <v>0.1825</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1885,7 +1885,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>0.2313</v>
+        <v>0.2325</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1910,7 +1910,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>1.2786</v>
+        <v>1.274</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -2010,7 +2010,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>1</v>
+        <v>0.95</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -2160,7 +2160,7 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>0.1649</v>
+        <v>0.1636</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2185,7 +2185,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>0.2344</v>
+        <v>0.2318</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2260,7 +2260,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>0.1577</v>
+        <v>0.1574</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2285,7 +2285,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>0.2228</v>
+        <v>0.2221</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2310,7 +2310,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>1.4128</v>
+        <v>1.4111</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2410,7 +2410,7 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>1</v>
+        <v>0.8205</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2810,7 +2810,7 @@
         </is>
       </c>
       <c r="D96" t="n">
-        <v>1</v>
+        <v>0.6571</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -3210,7 +3210,7 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>1</v>
+        <v>0.9077</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3360,7 +3360,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>0.1212</v>
+        <v>0.1171</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3385,7 +3385,7 @@
         </is>
       </c>
       <c r="D119" t="n">
-        <v>0.1923</v>
+        <v>0.1817</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3460,7 +3460,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>0.1289</v>
+        <v>0.1279</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3485,7 +3485,7 @@
         </is>
       </c>
       <c r="D123" t="n">
-        <v>0.1886</v>
+        <v>0.186</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3510,7 +3510,7 @@
         </is>
       </c>
       <c r="D124" t="n">
-        <v>1.4631</v>
+        <v>1.4543</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3610,7 +3610,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>1</v>
+        <v>0.9167</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3760,7 +3760,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>0.0128</v>
+        <v>0.0167</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3785,7 +3785,7 @@
         </is>
       </c>
       <c r="D135" t="n">
-        <v>0.0352</v>
+        <v>0.0435</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3860,7 +3860,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>0.0431</v>
+        <v>0.0441</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3885,7 +3885,7 @@
         </is>
       </c>
       <c r="D139" t="n">
-        <v>0.0806</v>
+        <v>0.08160000000000001</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3910,7 +3910,7 @@
         </is>
       </c>
       <c r="D140" t="n">
-        <v>1.8701</v>
+        <v>1.8503</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -4010,7 +4010,7 @@
         </is>
       </c>
       <c r="D144" t="n">
-        <v>1</v>
+        <v>0.9744</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -4410,7 +4410,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>1</v>
+        <v>0.9857</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4960,7 +4960,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>0.0417</v>
+        <v>0.0543</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4985,7 +4985,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>0.0635</v>
+        <v>0.0785</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -5060,7 +5060,7 @@
         </is>
       </c>
       <c r="D186" t="n">
-        <v>0.0528</v>
+        <v>0.0559</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -5085,7 +5085,7 @@
         </is>
       </c>
       <c r="D187" t="n">
-        <v>0.0887</v>
+        <v>0.0916</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5110,7 +5110,7 @@
         </is>
       </c>
       <c r="D188" t="n">
-        <v>1.6799</v>
+        <v>1.6386</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5210,7 +5210,7 @@
         </is>
       </c>
       <c r="D192" t="n">
-        <v>1</v>
+        <v>0.9333</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -7585,7 +7585,7 @@
         </is>
       </c>
       <c r="D287" t="n">
-        <v>0.1667</v>
+        <v>0.1648</v>
       </c>
       <c r="E287" t="inlineStr">
         <is>
@@ -7610,7 +7610,7 @@
         </is>
       </c>
       <c r="D288" t="n">
-        <v>0.2275</v>
+        <v>0.2245</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -7685,7 +7685,7 @@
         </is>
       </c>
       <c r="D291" t="n">
-        <v>0.2168</v>
+        <v>0.2163</v>
       </c>
       <c r="E291" t="inlineStr">
         <is>
@@ -7710,7 +7710,7 @@
         </is>
       </c>
       <c r="D292" t="n">
-        <v>0.2923</v>
+        <v>0.2917</v>
       </c>
       <c r="E292" t="inlineStr">
         <is>
@@ -7735,7 +7735,7 @@
         </is>
       </c>
       <c r="D293" t="n">
-        <v>1.3482</v>
+        <v>1.3486</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7835,7 +7835,7 @@
         </is>
       </c>
       <c r="D297" t="n">
-        <v>1</v>
+        <v>0.6974</v>
       </c>
       <c r="E297" t="inlineStr">
         <is>
@@ -8235,7 +8235,7 @@
         </is>
       </c>
       <c r="D313" t="n">
-        <v>1</v>
+        <v>0.6286</v>
       </c>
       <c r="E313" t="inlineStr">
         <is>
@@ -8635,7 +8635,7 @@
         </is>
       </c>
       <c r="D329" t="n">
-        <v>1</v>
+        <v>0.5846</v>
       </c>
       <c r="E329" t="inlineStr">
         <is>
@@ -8785,7 +8785,7 @@
         </is>
       </c>
       <c r="D335" t="n">
-        <v>0.1434</v>
+        <v>0.1375</v>
       </c>
       <c r="E335" t="inlineStr">
         <is>
@@ -8810,7 +8810,7 @@
         </is>
       </c>
       <c r="D336" t="n">
-        <v>0.2001</v>
+        <v>0.1887</v>
       </c>
       <c r="E336" t="inlineStr">
         <is>
@@ -8885,7 +8885,7 @@
         </is>
       </c>
       <c r="D339" t="n">
-        <v>0.1371</v>
+        <v>0.1356</v>
       </c>
       <c r="E339" t="inlineStr">
         <is>
@@ -8910,7 +8910,7 @@
         </is>
       </c>
       <c r="D340" t="n">
-        <v>0.186</v>
+        <v>0.183</v>
       </c>
       <c r="E340" t="inlineStr">
         <is>
@@ -8935,7 +8935,7 @@
         </is>
       </c>
       <c r="D341" t="n">
-        <v>1.3567</v>
+        <v>1.3496</v>
       </c>
       <c r="E341" t="inlineStr">
         <is>
@@ -9035,7 +9035,7 @@
         </is>
       </c>
       <c r="D345" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="E345" t="inlineStr">
         <is>
@@ -9185,7 +9185,7 @@
         </is>
       </c>
       <c r="D351" t="n">
-        <v>0.1358</v>
+        <v>0.134</v>
       </c>
       <c r="E351" t="inlineStr">
         <is>
@@ -9210,7 +9210,7 @@
         </is>
       </c>
       <c r="D352" t="n">
-        <v>0.2035</v>
+        <v>0.1993</v>
       </c>
       <c r="E352" t="inlineStr">
         <is>
@@ -9285,7 +9285,7 @@
         </is>
       </c>
       <c r="D355" t="n">
-        <v>0.1551</v>
+        <v>0.1546</v>
       </c>
       <c r="E355" t="inlineStr">
         <is>
@@ -9310,7 +9310,7 @@
         </is>
       </c>
       <c r="D356" t="n">
-        <v>0.2276</v>
+        <v>0.2267</v>
       </c>
       <c r="E356" t="inlineStr">
         <is>
@@ -9335,7 +9335,7 @@
         </is>
       </c>
       <c r="D357" t="n">
-        <v>1.4674</v>
+        <v>1.4664</v>
       </c>
       <c r="E357" t="inlineStr">
         <is>
@@ -9435,7 +9435,7 @@
         </is>
       </c>
       <c r="D361" t="n">
-        <v>1</v>
+        <v>0.7795</v>
       </c>
       <c r="E361" t="inlineStr">
         <is>
@@ -9835,7 +9835,7 @@
         </is>
       </c>
       <c r="D377" t="n">
-        <v>1</v>
+        <v>0.6286</v>
       </c>
       <c r="E377" t="inlineStr">
         <is>
@@ -10235,7 +10235,7 @@
         </is>
       </c>
       <c r="D393" t="n">
-        <v>1</v>
+        <v>0.7538</v>
       </c>
       <c r="E393" t="inlineStr">
         <is>
@@ -10385,7 +10385,7 @@
         </is>
       </c>
       <c r="D399" t="n">
-        <v>0.1129</v>
+        <v>0.1068</v>
       </c>
       <c r="E399" t="inlineStr">
         <is>
@@ -10410,7 +10410,7 @@
         </is>
       </c>
       <c r="D400" t="n">
-        <v>0.193</v>
+        <v>0.1782</v>
       </c>
       <c r="E400" t="inlineStr">
         <is>
@@ -10485,7 +10485,7 @@
         </is>
       </c>
       <c r="D403" t="n">
-        <v>0.1038</v>
+        <v>0.1023</v>
       </c>
       <c r="E403" t="inlineStr">
         <is>
@@ -10510,7 +10510,7 @@
         </is>
       </c>
       <c r="D404" t="n">
-        <v>0.1571</v>
+        <v>0.1527</v>
       </c>
       <c r="E404" t="inlineStr">
         <is>
@@ -10535,7 +10535,7 @@
         </is>
       </c>
       <c r="D405" t="n">
-        <v>1.5135</v>
+        <v>1.4927</v>
       </c>
       <c r="E405" t="inlineStr">
         <is>
@@ -10635,7 +10635,7 @@
         </is>
       </c>
       <c r="D409" t="n">
-        <v>1</v>
+        <v>0.9833</v>
       </c>
       <c r="E409" t="inlineStr">
         <is>
@@ -10785,7 +10785,7 @@
         </is>
       </c>
       <c r="D415" t="n">
-        <v>0.008500000000000001</v>
+        <v>0.0108</v>
       </c>
       <c r="E415" t="inlineStr">
         <is>
@@ -10810,7 +10810,7 @@
         </is>
       </c>
       <c r="D416" t="n">
-        <v>0.0356</v>
+        <v>0.0373</v>
       </c>
       <c r="E416" t="inlineStr">
         <is>
@@ -10885,7 +10885,7 @@
         </is>
       </c>
       <c r="D419" t="n">
-        <v>0.0471</v>
+        <v>0.0477</v>
       </c>
       <c r="E419" t="inlineStr">
         <is>
@@ -10910,7 +10910,7 @@
         </is>
       </c>
       <c r="D420" t="n">
-        <v>0.09909999999999999</v>
+        <v>0.0993</v>
       </c>
       <c r="E420" t="inlineStr">
         <is>
@@ -10935,7 +10935,7 @@
         </is>
       </c>
       <c r="D421" t="n">
-        <v>2.104</v>
+        <v>2.0818</v>
       </c>
       <c r="E421" t="inlineStr">
         <is>
@@ -11035,7 +11035,7 @@
         </is>
       </c>
       <c r="D425" t="n">
-        <v>1</v>
+        <v>0.9846</v>
       </c>
       <c r="E425" t="inlineStr">
         <is>
@@ -11985,7 +11985,7 @@
         </is>
       </c>
       <c r="D463" t="n">
-        <v>0.0271</v>
+        <v>0.0347</v>
       </c>
       <c r="E463" t="inlineStr">
         <is>
@@ -12010,7 +12010,7 @@
         </is>
       </c>
       <c r="D464" t="n">
-        <v>0.06419999999999999</v>
+        <v>0.0673</v>
       </c>
       <c r="E464" t="inlineStr">
         <is>
@@ -12085,7 +12085,7 @@
         </is>
       </c>
       <c r="D467" t="n">
-        <v>0.0479</v>
+        <v>0.0498</v>
       </c>
       <c r="E467" t="inlineStr">
         <is>
@@ -12110,7 +12110,7 @@
         </is>
       </c>
       <c r="D468" t="n">
-        <v>0.099</v>
+        <v>0.09959999999999999</v>
       </c>
       <c r="E468" t="inlineStr">
         <is>
@@ -12135,7 +12135,7 @@
         </is>
       </c>
       <c r="D469" t="n">
-        <v>2.0668</v>
+        <v>2</v>
       </c>
       <c r="E469" t="inlineStr">
         <is>
@@ -12235,7 +12235,7 @@
         </is>
       </c>
       <c r="D473" t="n">
-        <v>1</v>
+        <v>0.95</v>
       </c>
       <c r="E473" t="inlineStr">
         <is>
@@ -14610,7 +14610,7 @@
         </is>
       </c>
       <c r="D568" t="n">
-        <v>0.1679</v>
+        <v>0.169</v>
       </c>
       <c r="E568" t="inlineStr">
         <is>
@@ -14635,7 +14635,7 @@
         </is>
       </c>
       <c r="D569" t="n">
-        <v>0.2085</v>
+        <v>0.2084</v>
       </c>
       <c r="E569" t="inlineStr">
         <is>
@@ -14710,7 +14710,7 @@
         </is>
       </c>
       <c r="D572" t="n">
-        <v>0.23</v>
+        <v>0.2303</v>
       </c>
       <c r="E572" t="inlineStr">
         <is>
@@ -14760,7 +14760,7 @@
         </is>
       </c>
       <c r="D574" t="n">
-        <v>1.2596</v>
+        <v>1.2579</v>
       </c>
       <c r="E574" t="inlineStr">
         <is>
@@ -14860,7 +14860,7 @@
         </is>
       </c>
       <c r="D578" t="n">
-        <v>1</v>
+        <v>0.6513</v>
       </c>
       <c r="E578" t="inlineStr">
         <is>
@@ -15260,7 +15260,7 @@
         </is>
       </c>
       <c r="D594" t="n">
-        <v>1</v>
+        <v>0.7857</v>
       </c>
       <c r="E594" t="inlineStr">
         <is>
@@ -15660,7 +15660,7 @@
         </is>
       </c>
       <c r="D610" t="n">
-        <v>1</v>
+        <v>0.4923</v>
       </c>
       <c r="E610" t="inlineStr">
         <is>
@@ -15810,7 +15810,7 @@
         </is>
       </c>
       <c r="D616" t="n">
-        <v>0.1402</v>
+        <v>0.1437</v>
       </c>
       <c r="E616" t="inlineStr">
         <is>
@@ -15835,7 +15835,7 @@
         </is>
       </c>
       <c r="D617" t="n">
-        <v>0.1663</v>
+        <v>0.1661</v>
       </c>
       <c r="E617" t="inlineStr">
         <is>
@@ -15910,7 +15910,7 @@
         </is>
       </c>
       <c r="D620" t="n">
-        <v>0.2218</v>
+        <v>0.2226</v>
       </c>
       <c r="E620" t="inlineStr">
         <is>
@@ -15960,7 +15960,7 @@
         </is>
       </c>
       <c r="D622" t="n">
-        <v>1.2962</v>
+        <v>1.2916</v>
       </c>
       <c r="E622" t="inlineStr">
         <is>
@@ -16060,7 +16060,7 @@
         </is>
       </c>
       <c r="D626" t="n">
-        <v>1</v>
+        <v>0.6667</v>
       </c>
       <c r="E626" t="inlineStr">
         <is>
@@ -16210,7 +16210,7 @@
         </is>
       </c>
       <c r="D632" t="n">
-        <v>0.1391</v>
+        <v>0.1382</v>
       </c>
       <c r="E632" t="inlineStr">
         <is>
@@ -16235,7 +16235,7 @@
         </is>
       </c>
       <c r="D633" t="n">
-        <v>0.1957</v>
+        <v>0.1926</v>
       </c>
       <c r="E633" t="inlineStr">
         <is>
@@ -16310,7 +16310,7 @@
         </is>
       </c>
       <c r="D636" t="n">
-        <v>0.1547</v>
+        <v>0.1545</v>
       </c>
       <c r="E636" t="inlineStr">
         <is>
@@ -16335,7 +16335,7 @@
         </is>
       </c>
       <c r="D637" t="n">
-        <v>0.2203</v>
+        <v>0.2196</v>
       </c>
       <c r="E637" t="inlineStr">
         <is>
@@ -16360,7 +16360,7 @@
         </is>
       </c>
       <c r="D638" t="n">
-        <v>1.424</v>
+        <v>1.4214</v>
       </c>
       <c r="E638" t="inlineStr">
         <is>
@@ -16460,7 +16460,7 @@
         </is>
       </c>
       <c r="D642" t="n">
-        <v>1</v>
+        <v>0.7795</v>
       </c>
       <c r="E642" t="inlineStr">
         <is>
@@ -16860,7 +16860,7 @@
         </is>
       </c>
       <c r="D658" t="n">
-        <v>1</v>
+        <v>0.7857</v>
       </c>
       <c r="E658" t="inlineStr">
         <is>
@@ -17260,7 +17260,7 @@
         </is>
       </c>
       <c r="D674" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="E674" t="inlineStr">
         <is>
@@ -17410,7 +17410,7 @@
         </is>
       </c>
       <c r="D680" t="n">
-        <v>0.1019</v>
+        <v>0.099</v>
       </c>
       <c r="E680" t="inlineStr">
         <is>
@@ -17435,7 +17435,7 @@
         </is>
       </c>
       <c r="D681" t="n">
-        <v>0.1746</v>
+        <v>0.1633</v>
       </c>
       <c r="E681" t="inlineStr">
         <is>
@@ -17510,7 +17510,7 @@
         </is>
       </c>
       <c r="D684" t="n">
-        <v>0.1135</v>
+        <v>0.1128</v>
       </c>
       <c r="E684" t="inlineStr">
         <is>
@@ -17535,7 +17535,7 @@
         </is>
       </c>
       <c r="D685" t="n">
-        <v>0.1705</v>
+        <v>0.1676</v>
       </c>
       <c r="E685" t="inlineStr">
         <is>
@@ -17560,7 +17560,7 @@
         </is>
       </c>
       <c r="D686" t="n">
-        <v>1.5022</v>
+        <v>1.4858</v>
       </c>
       <c r="E686" t="inlineStr">
         <is>
@@ -17660,7 +17660,7 @@
         </is>
       </c>
       <c r="D690" t="n">
-        <v>1</v>
+        <v>0.9667</v>
       </c>
       <c r="E690" t="inlineStr">
         <is>
@@ -17810,7 +17810,7 @@
         </is>
       </c>
       <c r="D696" t="n">
-        <v>0.0086</v>
+        <v>0.0112</v>
       </c>
       <c r="E696" t="inlineStr">
         <is>
@@ -17835,7 +17835,7 @@
         </is>
       </c>
       <c r="D697" t="n">
-        <v>0.0348</v>
+        <v>0.0371</v>
       </c>
       <c r="E697" t="inlineStr">
         <is>
@@ -17910,7 +17910,7 @@
         </is>
       </c>
       <c r="D700" t="n">
-        <v>0.0463</v>
+        <v>0.047</v>
       </c>
       <c r="E700" t="inlineStr">
         <is>
@@ -17935,7 +17935,7 @@
         </is>
       </c>
       <c r="D701" t="n">
-        <v>0.08890000000000001</v>
+        <v>0.0891</v>
       </c>
       <c r="E701" t="inlineStr">
         <is>
@@ -17960,7 +17960,7 @@
         </is>
       </c>
       <c r="D702" t="n">
-        <v>1.9201</v>
+        <v>1.8957</v>
       </c>
       <c r="E702" t="inlineStr">
         <is>
@@ -18060,7 +18060,7 @@
         </is>
       </c>
       <c r="D706" t="n">
-        <v>1</v>
+        <v>0.9897</v>
       </c>
       <c r="E706" t="inlineStr">
         <is>
@@ -19010,7 +19010,7 @@
         </is>
       </c>
       <c r="D744" t="n">
-        <v>0.0279</v>
+        <v>0.0363</v>
       </c>
       <c r="E744" t="inlineStr">
         <is>
@@ -19035,7 +19035,7 @@
         </is>
       </c>
       <c r="D745" t="n">
-        <v>0.0626</v>
+        <v>0.0668</v>
       </c>
       <c r="E745" t="inlineStr">
         <is>
@@ -19110,7 +19110,7 @@
         </is>
       </c>
       <c r="D748" t="n">
-        <v>0.0396</v>
+        <v>0.0417</v>
       </c>
       <c r="E748" t="inlineStr">
         <is>
@@ -19135,7 +19135,7 @@
         </is>
       </c>
       <c r="D749" t="n">
-        <v>0.077</v>
+        <v>0.07779999999999999</v>
       </c>
       <c r="E749" t="inlineStr">
         <is>
@@ -19160,7 +19160,7 @@
         </is>
       </c>
       <c r="D750" t="n">
-        <v>1.9444</v>
+        <v>1.8657</v>
       </c>
       <c r="E750" t="inlineStr">
         <is>
@@ -19260,7 +19260,7 @@
         </is>
       </c>
       <c r="D754" t="n">
-        <v>1</v>
+        <v>0.9667</v>
       </c>
       <c r="E754" t="inlineStr">
         <is>
@@ -21635,7 +21635,7 @@
         </is>
       </c>
       <c r="D849" t="n">
-        <v>0.1829</v>
+        <v>0.1838</v>
       </c>
       <c r="E849" t="inlineStr">
         <is>
@@ -21660,7 +21660,7 @@
         </is>
       </c>
       <c r="D850" t="n">
-        <v>0.2341</v>
+        <v>0.233</v>
       </c>
       <c r="E850" t="inlineStr">
         <is>
@@ -21735,7 +21735,7 @@
         </is>
       </c>
       <c r="D853" t="n">
-        <v>0.2215</v>
+        <v>0.2217</v>
       </c>
       <c r="E853" t="inlineStr">
         <is>
@@ -21760,7 +21760,7 @@
         </is>
       </c>
       <c r="D854" t="n">
-        <v>0.2787</v>
+        <v>0.2785</v>
       </c>
       <c r="E854" t="inlineStr">
         <is>
@@ -21785,7 +21785,7 @@
         </is>
       </c>
       <c r="D855" t="n">
-        <v>1.2582</v>
+        <v>1.2562</v>
       </c>
       <c r="E855" t="inlineStr">
         <is>
@@ -21885,7 +21885,7 @@
         </is>
       </c>
       <c r="D859" t="n">
-        <v>1</v>
+        <v>0.641</v>
       </c>
       <c r="E859" t="inlineStr">
         <is>
@@ -22285,7 +22285,7 @@
         </is>
       </c>
       <c r="D875" t="n">
-        <v>1</v>
+        <v>0.6714</v>
       </c>
       <c r="E875" t="inlineStr">
         <is>
@@ -22685,7 +22685,7 @@
         </is>
       </c>
       <c r="D891" t="n">
-        <v>1</v>
+        <v>0.5846</v>
       </c>
       <c r="E891" t="inlineStr">
         <is>
@@ -22835,7 +22835,7 @@
         </is>
       </c>
       <c r="D897" t="n">
-        <v>0.1591</v>
+        <v>0.1621</v>
       </c>
       <c r="E897" t="inlineStr">
         <is>
@@ -22860,7 +22860,7 @@
         </is>
       </c>
       <c r="D898" t="n">
-        <v>0.2137</v>
+        <v>0.2099</v>
       </c>
       <c r="E898" t="inlineStr">
         <is>
@@ -22935,7 +22935,7 @@
         </is>
       </c>
       <c r="D901" t="n">
-        <v>0.193</v>
+        <v>0.1938</v>
       </c>
       <c r="E901" t="inlineStr">
         <is>
@@ -22960,7 +22960,7 @@
         </is>
       </c>
       <c r="D902" t="n">
-        <v>0.25</v>
+        <v>0.2492</v>
       </c>
       <c r="E902" t="inlineStr">
         <is>
@@ -22985,7 +22985,7 @@
         </is>
       </c>
       <c r="D903" t="n">
-        <v>1.2953</v>
+        <v>1.2859</v>
       </c>
       <c r="E903" t="inlineStr">
         <is>
@@ -23085,7 +23085,7 @@
         </is>
       </c>
       <c r="D907" t="n">
-        <v>1</v>
+        <v>0.6667</v>
       </c>
       <c r="E907" t="inlineStr">
         <is>
@@ -23235,7 +23235,7 @@
         </is>
       </c>
       <c r="D913" t="n">
-        <v>0.1759</v>
+        <v>0.1742</v>
       </c>
       <c r="E913" t="inlineStr">
         <is>
@@ -23260,7 +23260,7 @@
         </is>
       </c>
       <c r="D914" t="n">
-        <v>0.2419</v>
+        <v>0.2389</v>
       </c>
       <c r="E914" t="inlineStr">
         <is>
@@ -23335,7 +23335,7 @@
         </is>
       </c>
       <c r="D917" t="n">
-        <v>0.1752</v>
+        <v>0.1748</v>
       </c>
       <c r="E917" t="inlineStr">
         <is>
@@ -23360,7 +23360,7 @@
         </is>
       </c>
       <c r="D918" t="n">
-        <v>0.2344</v>
+        <v>0.2336</v>
       </c>
       <c r="E918" t="inlineStr">
         <is>
@@ -23385,7 +23385,7 @@
         </is>
       </c>
       <c r="D919" t="n">
-        <v>1.3379</v>
+        <v>1.3364</v>
       </c>
       <c r="E919" t="inlineStr">
         <is>
@@ -23485,7 +23485,7 @@
         </is>
       </c>
       <c r="D923" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="E923" t="inlineStr">
         <is>
@@ -23885,7 +23885,7 @@
         </is>
       </c>
       <c r="D939" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="E939" t="inlineStr">
         <is>
@@ -24285,7 +24285,7 @@
         </is>
       </c>
       <c r="D955" t="n">
-        <v>1</v>
+        <v>0.8615</v>
       </c>
       <c r="E955" t="inlineStr">
         <is>
@@ -24435,7 +24435,7 @@
         </is>
       </c>
       <c r="D961" t="n">
-        <v>0.1343</v>
+        <v>0.1288</v>
       </c>
       <c r="E961" t="inlineStr">
         <is>
@@ -24460,7 +24460,7 @@
         </is>
       </c>
       <c r="D962" t="n">
-        <v>0.2053</v>
+        <v>0.1934</v>
       </c>
       <c r="E962" t="inlineStr">
         <is>
@@ -24535,7 +24535,7 @@
         </is>
       </c>
       <c r="D965" t="n">
-        <v>0.1663</v>
+        <v>0.1649</v>
       </c>
       <c r="E965" t="inlineStr">
         <is>
@@ -24560,7 +24560,7 @@
         </is>
       </c>
       <c r="D966" t="n">
-        <v>0.2214</v>
+        <v>0.2187</v>
       </c>
       <c r="E966" t="inlineStr">
         <is>
@@ -24585,7 +24585,7 @@
         </is>
       </c>
       <c r="D967" t="n">
-        <v>1.3313</v>
+        <v>1.3263</v>
       </c>
       <c r="E967" t="inlineStr">
         <is>
@@ -24685,7 +24685,7 @@
         </is>
       </c>
       <c r="D971" t="n">
-        <v>1</v>
+        <v>0.7333</v>
       </c>
       <c r="E971" t="inlineStr">
         <is>
@@ -24835,7 +24835,7 @@
         </is>
       </c>
       <c r="D977" t="n">
-        <v>0.008399999999999999</v>
+        <v>0.0107</v>
       </c>
       <c r="E977" t="inlineStr">
         <is>
@@ -24860,7 +24860,7 @@
         </is>
       </c>
       <c r="D978" t="n">
-        <v>0.0356</v>
+        <v>0.0373</v>
       </c>
       <c r="E978" t="inlineStr">
         <is>
@@ -24935,7 +24935,7 @@
         </is>
       </c>
       <c r="D981" t="n">
-        <v>0.06759999999999999</v>
+        <v>0.0682</v>
       </c>
       <c r="E981" t="inlineStr">
         <is>
@@ -24960,7 +24960,7 @@
         </is>
       </c>
       <c r="D982" t="n">
-        <v>0.1525</v>
+        <v>0.1526</v>
       </c>
       <c r="E982" t="inlineStr">
         <is>
@@ -24985,7 +24985,7 @@
         </is>
       </c>
       <c r="D983" t="n">
-        <v>2.2559</v>
+        <v>2.2375</v>
       </c>
       <c r="E983" t="inlineStr">
         <is>
@@ -25085,7 +25085,7 @@
         </is>
       </c>
       <c r="D987" t="n">
-        <v>1</v>
+        <v>0.9641</v>
       </c>
       <c r="E987" t="inlineStr">
         <is>
@@ -25485,7 +25485,7 @@
         </is>
       </c>
       <c r="D1003" t="n">
-        <v>1</v>
+        <v>0.9714</v>
       </c>
       <c r="E1003" t="inlineStr">
         <is>
@@ -25885,7 +25885,7 @@
         </is>
       </c>
       <c r="D1019" t="n">
-        <v>1</v>
+        <v>0.9692</v>
       </c>
       <c r="E1019" t="inlineStr">
         <is>
@@ -26035,7 +26035,7 @@
         </is>
       </c>
       <c r="D1025" t="n">
-        <v>0.0271</v>
+        <v>0.0347</v>
       </c>
       <c r="E1025" t="inlineStr">
         <is>
@@ -26060,7 +26060,7 @@
         </is>
       </c>
       <c r="D1026" t="n">
-        <v>0.06419999999999999</v>
+        <v>0.0673</v>
       </c>
       <c r="E1026" t="inlineStr">
         <is>
@@ -26135,7 +26135,7 @@
         </is>
       </c>
       <c r="D1029" t="n">
-        <v>0.038</v>
+        <v>0.0399</v>
       </c>
       <c r="E1029" t="inlineStr">
         <is>
@@ -26160,7 +26160,7 @@
         </is>
       </c>
       <c r="D1030" t="n">
-        <v>0.0881</v>
+        <v>0.0887</v>
       </c>
       <c r="E1030" t="inlineStr">
         <is>
@@ -26185,7 +26185,7 @@
         </is>
       </c>
       <c r="D1031" t="n">
-        <v>2.3184</v>
+        <v>2.2231</v>
       </c>
       <c r="E1031" t="inlineStr">
         <is>
@@ -26285,7 +26285,7 @@
         </is>
       </c>
       <c r="D1035" t="n">
-        <v>1</v>
+        <v>0.95</v>
       </c>
       <c r="E1035" t="inlineStr">
         <is>

</xml_diff>